<commit_message>
Inherit FRCoreProcedureProfile directly from procedure-eu-core
Set Parent to procedure-eu-core (real FHIR inheritance, consistent with
FRCorePatientProfile/FRCorePractitionerProfile/FRCorePractitionerRoleProfile/
FRCoreOrganizationProfile) instead of documenting the EU Core link only in
a header comment. Drop the manual reasonReference restriction that
conflicted with the inherited target profile list (it now inherits
Condition EU Core/Observation/Procedure EU Core/DiagnosticReport/
DocumentReference directly); update comments to reflect what is now
inherited vs. still pending (FRCoreConditionProfile).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 3523e051d6402fbcd8a6ad82472de9b7533429fb
</commit_message>
<xml_diff>
--- a/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure-priority-extension.xlsx
+++ b/nr-doc-core-procedure/ig/StructureDefinition-fr-core-procedure-priority-extension.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T13:39:21+00:00</t>
+    <t>2026-07-22T12:47:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -347,7 +347,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActPriority-cisis|20260420150250</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActPriority-cisis|20260619134042</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}

</xml_diff>